<commit_message>
Update attendance: Etihad Altéa DCS training Oct 12-16
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_october_2026.xlsx
+++ b/omar_elnemr_attendance_october_2026.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1020,12 +1020,12 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:55 AM / Logged out 05:05 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 05:05 PM)</t>
         </is>
       </c>
     </row>
@@ -1060,12 +1060,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1140,23 +1140,63 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>07:55 AM</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>12:13 PM</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>4h 18m</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Training / Paid</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 12:13 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Total October Hours</t>
         </is>
       </c>
-      <c r="F18" s="12">
-        <f>SUM(F2:F16)</f>
+      <c r="F19" s="12">
+        <f>SUM(F2:F17)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Oct 16 log-out to 12:30 PM (4h 35m)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_october_2026.xlsx
+++ b/omar_elnemr_attendance_october_2026.xlsx
@@ -1167,16 +1167,16 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>12:13 PM</t>
+          <t>12:30 PM</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>4h 18m</t>
+          <t>4h 35m</t>
         </is>
       </c>
       <c r="F17" s="9" t="n">
-        <v>4.3</v>
+        <v>4.58</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 12:13 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 12:30 PM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update personal attendance: add September tab, fix Oct 9 status, and refine Oct 5-6 training notes
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_october_2026.xlsx
+++ b/omar_elnemr_attendance_october_2026.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Omar October 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="October 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="September 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -749,7 +750,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -789,7 +790,7 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -902,7 +903,11 @@
       <c r="F10" s="3" t="n">
         <v>9.380000000000001</v>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
           <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 05:13 PM)</t>
@@ -1192,11 +1197,408 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Total October Hours</t>
+          <t>Total October 2026 Hours</t>
         </is>
       </c>
       <c r="F19" s="12">
         <f>SUM(F2:F17)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="75" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Log-In</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Log-Out</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Decimal Hours</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>06:30 AM</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Standardized</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Standardized 23rd shift: 06:30 AM – 04:00 PM (9.5h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>08:15 AM</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>7h 45m</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Standard daytime shift</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>08:15 AM</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>9h 25m</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Overtime</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>⚡ Extended shift (+1h 40m overtime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>08:15 AM</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>7h 45m</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Standard daytime shift</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>08:15 AM</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>7h 45m</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Standard daytime shift (4:00 PM return)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>08:15 AM</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>7h 45m</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Standard daytime shift (4:00 PM return)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>08:15 AM</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>7h 45m</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Standard daytime shift (4:00 PM return)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Total September 2026 Hours</t>
+        </is>
+      </c>
+      <c r="F11" s="12">
+        <f>SUM(F2:F9)</f>
         <v/>
       </c>
     </row>

</xml_diff>